<commit_message>
fix(precio): la comparación de coste cuadra con 1.300 €
- Administrativo en España ≈ 2.700 €/mes (antes 2.500): con 1.300 € el ahorro
  es del 52 %, que es lo que dice la portada. Con 2.500 era un 48 %. Misma
  referencia que el vídeo de Meta v7f3. Portada y /asistente-virtual.
- Calculadora en Excel: el perfil Junior pasa de 1.200 a 1.300 €/mes. Editado
  directo en el XML para no perder el gráfico; recalcula al abrir.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Calculadora-de-Ahorro-Estrategico-GTC.xlsx
+++ b/public/Calculadora-de-Ahorro-Estrategico-GTC.xlsx
@@ -7,7 +7,7 @@
     <sheet state="visible" name="🧮 Calculadora" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -3514,7 +3514,7 @@
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="56">
-        <f>IF(C11="Junior",1200*12,IF(C11="Mid",1400*12,IF(C11="Senior",1650*12,0)))</f>
+        <f>IF(C11="Junior",1300*12,IF(C11="Mid",1400*12,IF(C11="Senior",1650*12,0)))</f>
         <v>19800</v>
       </c>
       <c r="G15" s="57">

</xml_diff>

<commit_message>
fix(precio): la comparación de coste cuadra con 1.300 € (#56)
- Administrativo en España ≈ 2.700 €/mes (antes 2.500): con 1.300 € el ahorro
  es del 52 %, que es lo que dice la portada. Con 2.500 era un 48 %. Misma
  referencia que el vídeo de Meta v7f3. Portada y /asistente-virtual.
- Calculadora en Excel: el perfil Junior pasa de 1.200 a 1.300 €/mes. Editado
  directo en el XML para no perder el gráfico; recalcula al abrir.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Calculadora-de-Ahorro-Estrategico-GTC.xlsx
+++ b/public/Calculadora-de-Ahorro-Estrategico-GTC.xlsx
@@ -7,7 +7,7 @@
     <sheet state="visible" name="🧮 Calculadora" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -3514,7 +3514,7 @@
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="56">
-        <f>IF(C11="Junior",1200*12,IF(C11="Mid",1400*12,IF(C11="Senior",1650*12,0)))</f>
+        <f>IF(C11="Junior",1300*12,IF(C11="Mid",1400*12,IF(C11="Senior",1650*12,0)))</f>
         <v>19800</v>
       </c>
       <c r="G15" s="57">

</xml_diff>